<commit_message>
feat: add Q9 boundary and BDS listings for Q9 + Binh Chanh
- Add Quan 9 (cu) boundary polygon to tphcm-districts.json
- Scrape and merge 6 new projects (2 Q9, 4 Binh Chanh) into 59 total
- Regenerate index.html map with 23 district polygons
- Regenerate chung_cu_data.xlsx with all 59 projects
- Add Q.9 color support to generate_excel.py
</commit_message>
<xml_diff>
--- a/chung_cu_data.xlsx
+++ b/chung_cu_data.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toa Do (Map)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh Sach BDS'!$A$1:$K$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh Sach BDS'!$A$1:$K$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -39,7 +39,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +88,18 @@
         <bgColor rgb="00E0F2F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3E5F5"/>
+        <bgColor rgb="00F3E5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFEBE9"/>
+        <bgColor rgb="00EFEBE9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -115,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -150,6 +162,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -516,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3400,8 +3422,338 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="20" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="21" t="inlineStr">
+        <is>
+          <t>The Origami (Vinhomes Grand Park)</t>
+        </is>
+      </c>
+      <c r="C55" s="21" t="inlineStr">
+        <is>
+          <t>Chung cu</t>
+        </is>
+      </c>
+      <c r="D55" s="21" t="inlineStr">
+        <is>
+          <t>3.3-4.9 ty</t>
+        </is>
+      </c>
+      <c r="E55" s="21" t="inlineStr">
+        <is>
+          <t>59-90m2</t>
+        </is>
+      </c>
+      <c r="F55" s="20" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="G55" s="20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H55" s="21" t="inlineStr">
+        <is>
+          <t>Long Binh, TP.Thu Duc (Q.9 cu)</t>
+        </is>
+      </c>
+      <c r="I55" s="21" t="inlineStr">
+        <is>
+          <t>Q.9</t>
+        </is>
+      </c>
+      <c r="J55" s="21" t="inlineStr">
+        <is>
+          <t>Vinhomes, view vuon Nhat, ho ca Koi</t>
+        </is>
+      </c>
+      <c r="K55" s="22" t="inlineStr">
+        <is>
+          <t>Xem BDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="20" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="21" t="inlineStr">
+        <is>
+          <t>Lumiere Boulevard</t>
+        </is>
+      </c>
+      <c r="C56" s="21" t="inlineStr">
+        <is>
+          <t>Chung cu</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="inlineStr">
+        <is>
+          <t>4.6-4.7 ty</t>
+        </is>
+      </c>
+      <c r="E56" s="21" t="inlineStr">
+        <is>
+          <t>74m2</t>
+        </is>
+      </c>
+      <c r="F56" s="20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G56" s="20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H56" s="21" t="inlineStr">
+        <is>
+          <t>Long Binh, TP.Thu Duc (Q.9 cu)</t>
+        </is>
+      </c>
+      <c r="I56" s="21" t="inlineStr">
+        <is>
+          <t>Q.9</t>
+        </is>
+      </c>
+      <c r="J56" s="21" t="inlineStr">
+        <is>
+          <t>Masterise Homes, trong Vinhomes GP</t>
+        </is>
+      </c>
+      <c r="K56" s="22" t="inlineStr">
+        <is>
+          <t>Xem BDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="23" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="24" t="inlineStr">
+        <is>
+          <t>Mizuki Park</t>
+        </is>
+      </c>
+      <c r="C57" s="24" t="inlineStr">
+        <is>
+          <t>Chung cu</t>
+        </is>
+      </c>
+      <c r="D57" s="24" t="inlineStr">
+        <is>
+          <t>3.6-4.2 ty</t>
+        </is>
+      </c>
+      <c r="E57" s="24" t="inlineStr">
+        <is>
+          <t>58-95m2</t>
+        </is>
+      </c>
+      <c r="F57" s="23" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="G57" s="23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H57" s="24" t="inlineStr">
+        <is>
+          <t>Nguyen Van Linh, X.Binh Hung, Binh Chanh</t>
+        </is>
+      </c>
+      <c r="I57" s="24" t="inlineStr">
+        <is>
+          <t>Binh Chanh</t>
+        </is>
+      </c>
+      <c r="J57" s="24" t="inlineStr">
+        <is>
+          <t>Nam Long, view song, khu do thi</t>
+        </is>
+      </c>
+      <c r="K57" s="25" t="inlineStr">
+        <is>
+          <t>Xem BDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="23" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="24" t="inlineStr">
+        <is>
+          <t>Trellia Cove (Mizuki Park)</t>
+        </is>
+      </c>
+      <c r="C58" s="24" t="inlineStr">
+        <is>
+          <t>Chung cu</t>
+        </is>
+      </c>
+      <c r="D58" s="24" t="inlineStr">
+        <is>
+          <t>3.9-5 ty</t>
+        </is>
+      </c>
+      <c r="E58" s="24" t="inlineStr">
+        <is>
+          <t>59-79m2</t>
+        </is>
+      </c>
+      <c r="F58" s="23" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="G58" s="23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H58" s="24" t="inlineStr">
+        <is>
+          <t>Nguyen Van Linh, X.Binh Hung, Binh Chanh</t>
+        </is>
+      </c>
+      <c r="I58" s="24" t="inlineStr">
+        <is>
+          <t>Binh Chanh</t>
+        </is>
+      </c>
+      <c r="J58" s="24" t="inlineStr">
+        <is>
+          <t>Nam Long, phan khu moi Mizuki Park</t>
+        </is>
+      </c>
+      <c r="K58" s="25" t="inlineStr">
+        <is>
+          <t>Xem BDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="23" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="24" t="inlineStr">
+        <is>
+          <t>Westgate An Gia</t>
+        </is>
+      </c>
+      <c r="C59" s="24" t="inlineStr">
+        <is>
+          <t>Chung cu</t>
+        </is>
+      </c>
+      <c r="D59" s="24" t="inlineStr">
+        <is>
+          <t>3.2-4.5 ty</t>
+        </is>
+      </c>
+      <c r="E59" s="24" t="inlineStr">
+        <is>
+          <t>59-113m2</t>
+        </is>
+      </c>
+      <c r="F59" s="23" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="G59" s="23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H59" s="24" t="inlineStr">
+        <is>
+          <t>Nguyen Van Linh, TT.Tan Tuc, Binh Chanh</t>
+        </is>
+      </c>
+      <c r="I59" s="24" t="inlineStr">
+        <is>
+          <t>Binh Chanh</t>
+        </is>
+      </c>
+      <c r="J59" s="24" t="inlineStr">
+        <is>
+          <t>An Gia Investment, so hong</t>
+        </is>
+      </c>
+      <c r="K59" s="25" t="inlineStr">
+        <is>
+          <t>Xem BDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="23" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="24" t="inlineStr">
+        <is>
+          <t>Sai Gon Mia</t>
+        </is>
+      </c>
+      <c r="C60" s="24" t="inlineStr">
+        <is>
+          <t>Chung cu</t>
+        </is>
+      </c>
+      <c r="D60" s="24" t="inlineStr">
+        <is>
+          <t>3.4-5 ty</t>
+        </is>
+      </c>
+      <c r="E60" s="24" t="inlineStr">
+        <is>
+          <t>66-78m2</t>
+        </is>
+      </c>
+      <c r="F60" s="23" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="G60" s="23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H60" s="24" t="inlineStr">
+        <is>
+          <t>Trung Son, X.Binh Hung, Binh Chanh</t>
+        </is>
+      </c>
+      <c r="I60" s="24" t="inlineStr">
+        <is>
+          <t>Binh Chanh</t>
+        </is>
+      </c>
+      <c r="J60" s="24" t="inlineStr">
+        <is>
+          <t>Hung Thinh, full noi that, view song</t>
+        </is>
+      </c>
+      <c r="K60" s="25" t="inlineStr">
+        <is>
+          <t>Xem BDS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K54"/>
+  <autoFilter ref="A1:K60"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -3456,6 +3808,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3467,7 +3825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3511,1486 +3869,1654 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>Topaz Elite</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B2" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C2" s="20" t="n">
+      <c r="C2" s="26" t="n">
         <v>10.7392189</v>
       </c>
-      <c r="D2" s="20" t="n">
+      <c r="D2" s="26" t="n">
         <v>106.6797322</v>
       </c>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="E2" s="26" t="inlineStr">
         <is>
           <t>3.2-4.8 ty</t>
         </is>
       </c>
-      <c r="F2" s="20" t="inlineStr">
+      <c r="F2" s="26" t="inlineStr">
         <is>
           <t>Cao Lo, P.4, Q.8</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>Topaz City</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C3" s="20" t="n">
+      <c r="C3" s="26" t="n">
         <v>10.7386</v>
       </c>
-      <c r="D3" s="20" t="n">
+      <c r="D3" s="26" t="n">
         <v>106.6798</v>
       </c>
-      <c r="E3" s="20" t="inlineStr">
+      <c r="E3" s="26" t="inlineStr">
         <is>
           <t>3.0-4.5 ty</t>
         </is>
       </c>
-      <c r="F3" s="20" t="inlineStr">
+      <c r="F3" s="26" t="inlineStr">
         <is>
           <t>Ta Quang Buu, P.5, Q.8</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>The Pegasuite</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="26" t="n">
         <v>10.7342516</v>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="26" t="n">
         <v>106.6533069</v>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="26" t="inlineStr">
         <is>
           <t>3.0-4.5 ty</t>
         </is>
       </c>
-      <c r="F4" s="20" t="inlineStr">
+      <c r="F4" s="26" t="inlineStr">
         <is>
           <t>Ta Quang Buu, P.6, Q.8</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>The Pegasuite 2</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="26" t="n">
         <v>10.7327</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="26" t="n">
         <v>106.6501</v>
       </c>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>3.2-5.0 ty</t>
         </is>
       </c>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Ta Quang Buu, P.6, Q.8</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>D-Aqua</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="26" t="n">
         <v>10.7402309</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="26" t="n">
         <v>106.645793</v>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="E6" s="26" t="inlineStr">
         <is>
           <t>3.5-5.0 ty</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="26" t="inlineStr">
         <is>
           <t>Ben Binh Dong, P.14, Q.8</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Aurora Residences</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="26" t="n">
         <v>10.7429092</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="26" t="n">
         <v>106.6508679</v>
       </c>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="E7" s="26" t="inlineStr">
         <is>
           <t>3.0-4.5 ty</t>
         </is>
       </c>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="F7" s="26" t="inlineStr">
         <is>
           <t>Ben Binh Dong, P.13, Q.8</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Green River</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="26" t="n">
         <v>10.7335</v>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="26" t="n">
         <v>106.6442</v>
       </c>
-      <c r="E8" s="20" t="inlineStr">
+      <c r="E8" s="26" t="inlineStr">
         <is>
           <t>3.0-3.8 ty</t>
         </is>
       </c>
-      <c r="F8" s="20" t="inlineStr">
+      <c r="F8" s="26" t="inlineStr">
         <is>
           <t>Pham The Hien, P.7, Q.8</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Tara Residence</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="26" t="n">
         <v>10.7325</v>
       </c>
-      <c r="D9" s="20" t="n">
+      <c r="D9" s="26" t="n">
         <v>106.6531</v>
       </c>
-      <c r="E9" s="20" t="inlineStr">
+      <c r="E9" s="26" t="inlineStr">
         <is>
           <t>3.0-4.2 ty</t>
         </is>
       </c>
-      <c r="F9" s="20" t="inlineStr">
+      <c r="F9" s="26" t="inlineStr">
         <is>
           <t>Ta Quang Buu, P.6, Q.8</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Saigon Skyview</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="26" t="n">
         <v>10.7328855</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="26" t="n">
         <v>106.6557022</v>
       </c>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="E10" s="26" t="inlineStr">
         <is>
           <t>3.0-4.5 ty</t>
         </is>
       </c>
-      <c r="F10" s="20" t="inlineStr">
+      <c r="F10" s="26" t="inlineStr">
         <is>
           <t>Ta Quang Buu, P.6, Q.8</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>Central Premium</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="26" t="n">
         <v>10.7369</v>
       </c>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="26" t="n">
         <v>106.6691</v>
       </c>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="E11" s="26" t="inlineStr">
         <is>
           <t>3.5-5.0 ty</t>
         </is>
       </c>
-      <c r="F11" s="20" t="inlineStr">
+      <c r="F11" s="26" t="inlineStr">
         <is>
           <t>Ta Quang Buu, P.1, Q.8</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>CC Bong Sao</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="26" t="n">
         <v>10.7368621</v>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="D12" s="26" t="n">
         <v>106.6613181</v>
       </c>
-      <c r="E12" s="20" t="inlineStr">
+      <c r="E12" s="26" t="inlineStr">
         <is>
           <t>3.0-3.5 ty</t>
         </is>
       </c>
-      <c r="F12" s="20" t="inlineStr">
+      <c r="F12" s="26" t="inlineStr">
         <is>
           <t>Ta Quang Buu, P.5, Q.8</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t>Diamond Riverside</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="26" t="n">
         <v>10.7302</v>
       </c>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="26" t="n">
         <v>106.6248</v>
       </c>
-      <c r="E13" s="20" t="inlineStr">
+      <c r="E13" s="26" t="inlineStr">
         <is>
           <t>3.0-4.0 ty</t>
         </is>
       </c>
-      <c r="F13" s="20" t="inlineStr">
+      <c r="F13" s="26" t="inlineStr">
         <is>
           <t>Vo Van Kiet, P.16, Q.8</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Conic Riverside</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>Q.8</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="26" t="n">
         <v>10.7184884</v>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="26" t="n">
         <v>106.6371053</v>
       </c>
-      <c r="E14" s="20" t="inlineStr">
+      <c r="E14" s="26" t="inlineStr">
         <is>
           <t>3.0-4.2 ty</t>
         </is>
       </c>
-      <c r="F14" s="20" t="inlineStr">
+      <c r="F14" s="26" t="inlineStr">
         <is>
           <t>Ta Quang Buu, P.7, Q.8</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Asiana Capella</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="26" t="inlineStr">
         <is>
           <t>Q.6</t>
         </is>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="26" t="n">
         <v>10.7398895</v>
       </c>
-      <c r="D15" s="20" t="n">
+      <c r="D15" s="26" t="n">
         <v>106.6280712</v>
       </c>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="E15" s="26" t="inlineStr">
         <is>
           <t>3.5-5.0 ty</t>
         </is>
       </c>
-      <c r="F15" s="20" t="inlineStr">
+      <c r="F15" s="26" t="inlineStr">
         <is>
           <t>Tran Van Kieu, P.10, Q.6</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>Him Lam Cho Lon</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>Q.6</t>
         </is>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="26" t="n">
         <v>10.7466</v>
       </c>
-      <c r="D16" s="20" t="n">
+      <c r="D16" s="26" t="n">
         <v>106.6379</v>
       </c>
-      <c r="E16" s="20" t="inlineStr">
+      <c r="E16" s="26" t="inlineStr">
         <is>
           <t>3.0-4.5 ty</t>
         </is>
       </c>
-      <c r="F16" s="20" t="inlineStr">
+      <c r="F16" s="26" t="inlineStr">
         <is>
           <t>Dai lo Dong Tay, P.11, Q.6</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t>Viva Riverside</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>Q.6</t>
         </is>
       </c>
-      <c r="C17" s="20" t="n">
+      <c r="C17" s="26" t="n">
         <v>10.7427112</v>
       </c>
-      <c r="D17" s="20" t="n">
+      <c r="D17" s="26" t="n">
         <v>106.6474475</v>
       </c>
-      <c r="E17" s="20" t="inlineStr">
+      <c r="E17" s="26" t="inlineStr">
         <is>
           <t>3.0-4.5 ty</t>
         </is>
       </c>
-      <c r="F17" s="20" t="inlineStr">
+      <c r="F17" s="26" t="inlineStr">
         <is>
           <t>Vo Van Kiet, P.1, Q.6</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>Saigon Asiana</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="26" t="inlineStr">
         <is>
           <t>Q.6</t>
         </is>
       </c>
-      <c r="C18" s="20" t="n">
+      <c r="C18" s="26" t="n">
         <v>10.7501021</v>
       </c>
-      <c r="D18" s="20" t="n">
+      <c r="D18" s="26" t="n">
         <v>106.6367849</v>
       </c>
-      <c r="E18" s="20" t="inlineStr">
+      <c r="E18" s="26" t="inlineStr">
         <is>
           <t>3.0-4.2 ty</t>
         </is>
       </c>
-      <c r="F18" s="20" t="inlineStr">
+      <c r="F18" s="26" t="inlineStr">
         <is>
           <t>NV Luong, P.12, Q.6</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>D-Homme</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>Q.6</t>
         </is>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="26" t="n">
         <v>10.7537</v>
       </c>
-      <c r="D19" s="20" t="n">
+      <c r="D19" s="26" t="n">
         <v>106.6446</v>
       </c>
-      <c r="E19" s="20" t="inlineStr">
+      <c r="E19" s="26" t="inlineStr">
         <is>
           <t>3.8-5.0 ty</t>
         </is>
       </c>
-      <c r="F19" s="20" t="inlineStr">
+      <c r="F19" s="26" t="inlineStr">
         <is>
           <t>Hong Bang, P.12, Q.6</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A20" s="26" t="inlineStr">
         <is>
           <t>Summer Square</t>
         </is>
       </c>
-      <c r="B20" s="20" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>Q.6</t>
         </is>
       </c>
-      <c r="C20" s="20" t="n">
+      <c r="C20" s="26" t="n">
         <v>10.7593879</v>
       </c>
-      <c r="D20" s="20" t="n">
+      <c r="D20" s="26" t="n">
         <v>106.6259582</v>
       </c>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="E20" s="26" t="inlineStr">
         <is>
           <t>3.0-3.8 ty</t>
         </is>
       </c>
-      <c r="F20" s="20" t="inlineStr">
+      <c r="F20" s="26" t="inlineStr">
         <is>
           <t>Tan Hoa Dong, P.14, Q.6</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>CHCC 155 Nguyen Chi Thanh</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B21" s="26" t="inlineStr">
         <is>
           <t>Q.5</t>
         </is>
       </c>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="26" t="n">
         <v>10.7811842</v>
       </c>
-      <c r="D21" s="20" t="n">
+      <c r="D21" s="26" t="n">
         <v>106.7060405</v>
       </c>
-      <c r="E21" s="20" t="inlineStr">
+      <c r="E21" s="26" t="inlineStr">
         <is>
           <t>4.3 ty</t>
         </is>
       </c>
-      <c r="F21" s="20" t="inlineStr">
+      <c r="F21" s="26" t="inlineStr">
         <is>
           <t>155 Nguyen Chi Thanh, P.9, Q.5</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="20" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>Chung cu Hung Vuong (Tan Da)</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B22" s="26" t="inlineStr">
         <is>
           <t>Q.5</t>
         </is>
       </c>
-      <c r="C22" s="20" t="n">
+      <c r="C22" s="26" t="n">
         <v>10.7538946</v>
       </c>
-      <c r="D22" s="20" t="n">
+      <c r="D22" s="26" t="n">
         <v>106.6653437</v>
       </c>
-      <c r="E22" s="20" t="inlineStr">
+      <c r="E22" s="26" t="inlineStr">
         <is>
           <t>3.05-3.2 ty</t>
         </is>
       </c>
-      <c r="F22" s="20" t="inlineStr">
+      <c r="F22" s="26" t="inlineStr">
         <is>
           <t>Tan Da, P.11, Q.5</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>Chung cu Nguyen Trai</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B23" s="26" t="inlineStr">
         <is>
           <t>Q.5</t>
         </is>
       </c>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="26" t="n">
         <v>10.7557827</v>
       </c>
-      <c r="D23" s="20" t="n">
+      <c r="D23" s="26" t="n">
         <v>106.6690391</v>
       </c>
-      <c r="E23" s="20" t="inlineStr">
+      <c r="E23" s="26" t="inlineStr">
         <is>
           <t>3.25 ty</t>
         </is>
       </c>
-      <c r="F23" s="20" t="inlineStr">
+      <c r="F23" s="26" t="inlineStr">
         <is>
           <t>Nguyen Trai, P.1, Q.5</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="A24" s="26" t="inlineStr">
         <is>
           <t>The Everrich Infinity</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B24" s="26" t="inlineStr">
         <is>
           <t>Q.5</t>
         </is>
       </c>
-      <c r="C24" s="20" t="n">
+      <c r="C24" s="26" t="n">
         <v>10.760861</v>
       </c>
-      <c r="D24" s="20" t="n">
+      <c r="D24" s="26" t="n">
         <v>106.6806479</v>
       </c>
-      <c r="E24" s="20" t="inlineStr">
+      <c r="E24" s="26" t="inlineStr">
         <is>
           <t>3.3-4.5 ty</t>
         </is>
       </c>
-      <c r="F24" s="20" t="inlineStr">
+      <c r="F24" s="26" t="inlineStr">
         <is>
           <t>An Duong Vuong, P.4, Q.5</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="inlineStr">
+      <c r="A25" s="26" t="inlineStr">
         <is>
           <t>Can ho Lakai</t>
         </is>
       </c>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B25" s="26" t="inlineStr">
         <is>
           <t>Q.5</t>
         </is>
       </c>
-      <c r="C25" s="20" t="n">
+      <c r="C25" s="26" t="n">
         <v>10.7540121</v>
       </c>
-      <c r="D25" s="20" t="n">
+      <c r="D25" s="26" t="n">
         <v>106.6697165</v>
       </c>
-      <c r="E25" s="20" t="inlineStr">
+      <c r="E25" s="26" t="inlineStr">
         <is>
           <t>4.4 ty</t>
         </is>
       </c>
-      <c r="F25" s="20" t="inlineStr">
+      <c r="F25" s="26" t="inlineStr">
         <is>
           <t>Nguyen Tri Phuong, P.8, Q.5</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="20" t="inlineStr">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t>Legacy 66 Tan Thanh</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B26" s="26" t="inlineStr">
         <is>
           <t>Q.5</t>
         </is>
       </c>
-      <c r="C26" s="20" t="n">
+      <c r="C26" s="26" t="n">
         <v>10.7564974</v>
       </c>
-      <c r="D26" s="20" t="n">
+      <c r="D26" s="26" t="n">
         <v>106.6565336</v>
       </c>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="E26" s="26" t="inlineStr">
         <is>
           <t>4.5 ty</t>
         </is>
       </c>
-      <c r="F26" s="20" t="inlineStr">
+      <c r="F26" s="26" t="inlineStr">
         <is>
           <t>Tan Thanh, P.12, Q.5</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="20" t="inlineStr">
+      <c r="A27" s="26" t="inlineStr">
         <is>
           <t>CC Phan Van Tri Q5</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B27" s="26" t="inlineStr">
         <is>
           <t>Q.5</t>
         </is>
       </c>
-      <c r="C27" s="20" t="n">
+      <c r="C27" s="26" t="n">
         <v>10.7535</v>
       </c>
-      <c r="D27" s="20" t="n">
+      <c r="D27" s="26" t="n">
         <v>106.6723</v>
       </c>
-      <c r="E27" s="20" t="inlineStr">
+      <c r="E27" s="26" t="inlineStr">
         <is>
           <t>3.15 ty</t>
         </is>
       </c>
-      <c r="F27" s="20" t="inlineStr">
+      <c r="F27" s="26" t="inlineStr">
         <is>
           <t>Phan Van Tri, P.2, Q.5</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="20" t="inlineStr">
+      <c r="A28" s="26" t="inlineStr">
         <is>
           <t>Chung cu Phuc Thinh</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B28" s="26" t="inlineStr">
         <is>
           <t>Q.5</t>
         </is>
       </c>
-      <c r="C28" s="20" t="n">
+      <c r="C28" s="26" t="n">
         <v>10.7534138</v>
       </c>
-      <c r="D28" s="20" t="n">
+      <c r="D28" s="26" t="n">
         <v>106.6802515</v>
       </c>
-      <c r="E28" s="20" t="inlineStr">
+      <c r="E28" s="26" t="inlineStr">
         <is>
           <t>3.75-4.6 ty</t>
         </is>
       </c>
-      <c r="F28" s="20" t="inlineStr">
+      <c r="F28" s="26" t="inlineStr">
         <is>
           <t>Cao Dat, P.1, Q.5</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="20" t="inlineStr">
+      <c r="A29" s="26" t="inlineStr">
         <is>
           <t>CC Dao Tan Q5</t>
         </is>
       </c>
-      <c r="B29" s="20" t="inlineStr">
+      <c r="B29" s="26" t="inlineStr">
         <is>
           <t>Q.5</t>
         </is>
       </c>
-      <c r="C29" s="20" t="n">
+      <c r="C29" s="26" t="n">
         <v>10.752</v>
       </c>
-      <c r="D29" s="20" t="n">
+      <c r="D29" s="26" t="n">
         <v>106.6697</v>
       </c>
-      <c r="E29" s="20" t="inlineStr">
+      <c r="E29" s="26" t="inlineStr">
         <is>
           <t>4.66 ty</t>
         </is>
       </c>
-      <c r="F29" s="20" t="inlineStr">
+      <c r="F29" s="26" t="inlineStr">
         <is>
           <t>Dao Tan, P.5, Q.5</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="20" t="inlineStr">
+      <c r="A30" s="26" t="inlineStr">
         <is>
           <t>CC Nguyen Bieu Q5</t>
         </is>
       </c>
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B30" s="26" t="inlineStr">
         <is>
           <t>Q.5</t>
         </is>
       </c>
-      <c r="C30" s="20" t="n">
+      <c r="C30" s="26" t="n">
         <v>10.7556705</v>
       </c>
-      <c r="D30" s="20" t="n">
+      <c r="D30" s="26" t="n">
         <v>106.6732042</v>
       </c>
-      <c r="E30" s="20" t="inlineStr">
+      <c r="E30" s="26" t="inlineStr">
         <is>
           <t>3 ty</t>
         </is>
       </c>
-      <c r="F30" s="20" t="inlineStr">
+      <c r="F30" s="26" t="inlineStr">
         <is>
           <t>Nguyen Bieu, P.1, Q.5</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="20" t="inlineStr">
+      <c r="A31" s="26" t="inlineStr">
         <is>
           <t>Chung cu Le Thi Rieng</t>
         </is>
       </c>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>Q.10</t>
         </is>
       </c>
-      <c r="C31" s="20" t="n">
+      <c r="C31" s="26" t="n">
         <v>10.7811901</v>
       </c>
-      <c r="D31" s="20" t="n">
+      <c r="D31" s="26" t="n">
         <v>106.6630125</v>
       </c>
-      <c r="E31" s="20" t="inlineStr">
+      <c r="E31" s="26" t="inlineStr">
         <is>
           <t>3.8 ty</t>
         </is>
       </c>
-      <c r="F31" s="20" t="inlineStr">
+      <c r="F31" s="26" t="inlineStr">
         <is>
           <t>Le Thi Rieng, P.15, Q.10</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="20" t="inlineStr">
+      <c r="A32" s="26" t="inlineStr">
         <is>
           <t>CC Ly Thuong Kiet Q10</t>
         </is>
       </c>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B32" s="26" t="inlineStr">
         <is>
           <t>Q.10</t>
         </is>
       </c>
-      <c r="C32" s="20" t="n">
+      <c r="C32" s="26" t="n">
         <v>10.768769</v>
       </c>
-      <c r="D32" s="20" t="n">
+      <c r="D32" s="26" t="n">
         <v>106.6617061</v>
       </c>
-      <c r="E32" s="20" t="inlineStr">
+      <c r="E32" s="26" t="inlineStr">
         <is>
           <t>3 ty</t>
         </is>
       </c>
-      <c r="F32" s="20" t="inlineStr">
+      <c r="F32" s="26" t="inlineStr">
         <is>
           <t>Ly Thuong Kiet, P.7, Q.10</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="20" t="inlineStr">
+      <c r="A33" s="26" t="inlineStr">
         <is>
           <t>Cao oc Ngo Gia Tu</t>
         </is>
       </c>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B33" s="26" t="inlineStr">
         <is>
           <t>Q.10</t>
         </is>
       </c>
-      <c r="C33" s="20" t="n">
+      <c r="C33" s="26" t="n">
         <v>10.7638244</v>
       </c>
-      <c r="D33" s="20" t="n">
+      <c r="D33" s="26" t="n">
         <v>106.6716585</v>
       </c>
-      <c r="E33" s="20" t="inlineStr">
+      <c r="E33" s="26" t="inlineStr">
         <is>
           <t>3.9 ty</t>
         </is>
       </c>
-      <c r="F33" s="20" t="inlineStr">
+      <c r="F33" s="26" t="inlineStr">
         <is>
           <t>Ngo Gia Tu, P.3, Q.10</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="20" t="inlineStr">
+      <c r="A34" s="26" t="inlineStr">
         <is>
           <t>Chung cu Nguyen Kim</t>
         </is>
       </c>
-      <c r="B34" s="20" t="inlineStr">
+      <c r="B34" s="26" t="inlineStr">
         <is>
           <t>Q.10</t>
         </is>
       </c>
-      <c r="C34" s="20" t="n">
+      <c r="C34" s="26" t="n">
         <v>10.7613175</v>
       </c>
-      <c r="D34" s="20" t="n">
+      <c r="D34" s="26" t="n">
         <v>106.6618954</v>
       </c>
-      <c r="E34" s="20" t="inlineStr">
+      <c r="E34" s="26" t="inlineStr">
         <is>
           <t>3.45 ty</t>
         </is>
       </c>
-      <c r="F34" s="20" t="inlineStr">
+      <c r="F34" s="26" t="inlineStr">
         <is>
           <t>Nguyen Kim, P.7, Q.10</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="20" t="inlineStr">
+      <c r="A35" s="26" t="inlineStr">
         <is>
           <t>Hoa Sen - Lotus Apartment</t>
         </is>
       </c>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>Q.11</t>
         </is>
       </c>
-      <c r="C35" s="20" t="n">
+      <c r="C35" s="26" t="n">
         <v>10.7660078</v>
       </c>
-      <c r="D35" s="20" t="n">
+      <c r="D35" s="26" t="n">
         <v>106.6427565</v>
       </c>
-      <c r="E35" s="20" t="inlineStr">
+      <c r="E35" s="26" t="inlineStr">
         <is>
           <t>4.3 ty</t>
         </is>
       </c>
-      <c r="F35" s="20" t="inlineStr">
+      <c r="F35" s="26" t="inlineStr">
         <is>
           <t>Lac Long Quan, P.10, Q.11</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+      <c r="A36" s="26" t="inlineStr">
         <is>
           <t>CC Ly Thuong Kiet Q11</t>
         </is>
       </c>
-      <c r="B36" s="20" t="inlineStr">
+      <c r="B36" s="26" t="inlineStr">
         <is>
           <t>Q.11</t>
         </is>
       </c>
-      <c r="C36" s="20" t="n">
+      <c r="C36" s="26" t="n">
         <v>10.7683972</v>
       </c>
-      <c r="D36" s="20" t="n">
+      <c r="D36" s="26" t="n">
         <v>106.6618361</v>
       </c>
-      <c r="E36" s="20" t="inlineStr">
+      <c r="E36" s="26" t="inlineStr">
         <is>
           <t>3.2 ty</t>
         </is>
       </c>
-      <c r="F36" s="20" t="inlineStr">
+      <c r="F36" s="26" t="inlineStr">
         <is>
           <t>Ly Thuong Kiet, P.7, Q.11</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="20" t="inlineStr">
+      <c r="A37" s="26" t="inlineStr">
         <is>
           <t>CC Lac Long Quan Q11</t>
         </is>
       </c>
-      <c r="B37" s="20" t="inlineStr">
+      <c r="B37" s="26" t="inlineStr">
         <is>
           <t>Q.11</t>
         </is>
       </c>
-      <c r="C37" s="20" t="n">
+      <c r="C37" s="26" t="n">
         <v>10.7706699</v>
       </c>
-      <c r="D37" s="20" t="n">
+      <c r="D37" s="26" t="n">
         <v>106.6443301</v>
       </c>
-      <c r="E37" s="20" t="inlineStr">
+      <c r="E37" s="26" t="inlineStr">
         <is>
           <t>3.63 ty</t>
         </is>
       </c>
-      <c r="F37" s="20" t="inlineStr">
+      <c r="F37" s="26" t="inlineStr">
         <is>
           <t>Lac Long Quan, P.5, Q.11</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="20" t="inlineStr">
+      <c r="A38" s="26" t="inlineStr">
         <is>
           <t>Res 11</t>
         </is>
       </c>
-      <c r="B38" s="20" t="inlineStr">
+      <c r="B38" s="26" t="inlineStr">
         <is>
           <t>Q.11</t>
         </is>
       </c>
-      <c r="C38" s="20" t="n">
+      <c r="C38" s="26" t="n">
         <v>10.763534</v>
       </c>
-      <c r="D38" s="20" t="n">
+      <c r="D38" s="26" t="n">
         <v>106.6419219</v>
       </c>
-      <c r="E38" s="20" t="inlineStr">
+      <c r="E38" s="26" t="inlineStr">
         <is>
           <t>3.55-5 ty</t>
         </is>
       </c>
-      <c r="F38" s="20" t="inlineStr">
+      <c r="F38" s="26" t="inlineStr">
         <is>
           <t>Lac Long Quan, P.3, Q.11</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="inlineStr">
+      <c r="A39" s="26" t="inlineStr">
         <is>
           <t>Chung cu 312 Lac Long Quan</t>
         </is>
       </c>
-      <c r="B39" s="20" t="inlineStr">
+      <c r="B39" s="26" t="inlineStr">
         <is>
           <t>Q.11</t>
         </is>
       </c>
-      <c r="C39" s="20" t="n">
+      <c r="C39" s="26" t="n">
         <v>10.7686327</v>
       </c>
-      <c r="D39" s="20" t="n">
+      <c r="D39" s="26" t="n">
         <v>106.644232</v>
       </c>
-      <c r="E39" s="20" t="inlineStr">
+      <c r="E39" s="26" t="inlineStr">
         <is>
           <t>3.4 ty</t>
         </is>
       </c>
-      <c r="F39" s="20" t="inlineStr">
+      <c r="F39" s="26" t="inlineStr">
         <is>
           <t>312 Lac Long Quan, P.5, Q.11</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="20" t="inlineStr">
+      <c r="A40" s="26" t="inlineStr">
         <is>
           <t>Chung cu Phu Tho Q11</t>
         </is>
       </c>
-      <c r="B40" s="20" t="inlineStr">
+      <c r="B40" s="26" t="inlineStr">
         <is>
           <t>Q.11</t>
         </is>
       </c>
-      <c r="C40" s="20" t="n">
+      <c r="C40" s="26" t="n">
         <v>10.7698821</v>
       </c>
-      <c r="D40" s="20" t="n">
+      <c r="D40" s="26" t="n">
         <v>106.6534079</v>
       </c>
-      <c r="E40" s="20" t="inlineStr">
+      <c r="E40" s="26" t="inlineStr">
         <is>
           <t>3.7 ty</t>
         </is>
       </c>
-      <c r="F40" s="20" t="inlineStr">
+      <c r="F40" s="26" t="inlineStr">
         <is>
           <t>Nguyen Thi Nho, P.15, Q.11</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="20" t="inlineStr">
+      <c r="A41" s="26" t="inlineStr">
         <is>
           <t>H3 Hoang Dieu</t>
         </is>
       </c>
-      <c r="B41" s="20" t="inlineStr">
+      <c r="B41" s="26" t="inlineStr">
         <is>
           <t>Q.4</t>
         </is>
       </c>
-      <c r="C41" s="20" t="n">
+      <c r="C41" s="26" t="n">
         <v>10.7603234</v>
       </c>
-      <c r="D41" s="20" t="n">
+      <c r="D41" s="26" t="n">
         <v>106.6990936</v>
       </c>
-      <c r="E41" s="20" t="inlineStr">
+      <c r="E41" s="26" t="inlineStr">
         <is>
           <t>4.3 ty</t>
         </is>
       </c>
-      <c r="F41" s="20" t="inlineStr">
+      <c r="F41" s="26" t="inlineStr">
         <is>
           <t>Hoang Dieu, P. Khanh Hoi, Q.4</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="20" t="inlineStr">
+      <c r="A42" s="26" t="inlineStr">
         <is>
           <t>Saigon Royal Residence</t>
         </is>
       </c>
-      <c r="B42" s="20" t="inlineStr">
+      <c r="B42" s="26" t="inlineStr">
         <is>
           <t>Q.4</t>
         </is>
       </c>
-      <c r="C42" s="20" t="n">
+      <c r="C42" s="26" t="n">
         <v>10.7670153</v>
       </c>
-      <c r="D42" s="20" t="n">
+      <c r="D42" s="26" t="n">
         <v>106.7038674</v>
       </c>
-      <c r="E42" s="20" t="inlineStr">
+      <c r="E42" s="26" t="inlineStr">
         <is>
           <t>4.3 ty</t>
         </is>
       </c>
-      <c r="F42" s="20" t="inlineStr">
+      <c r="F42" s="26" t="inlineStr">
         <is>
           <t>Ben Van Don, P. Xom Chieu, Q.4</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="20" t="inlineStr">
+      <c r="A43" s="26" t="inlineStr">
         <is>
           <t>The Gold View</t>
         </is>
       </c>
-      <c r="B43" s="20" t="inlineStr">
+      <c r="B43" s="26" t="inlineStr">
         <is>
           <t>Q.4</t>
         </is>
       </c>
-      <c r="C43" s="20" t="n">
+      <c r="C43" s="26" t="n">
         <v>10.756248</v>
       </c>
-      <c r="D43" s="20" t="n">
+      <c r="D43" s="26" t="n">
         <v>106.6918721</v>
       </c>
-      <c r="E43" s="20" t="inlineStr">
+      <c r="E43" s="26" t="inlineStr">
         <is>
           <t>3.2 ty</t>
         </is>
       </c>
-      <c r="F43" s="20" t="inlineStr">
+      <c r="F43" s="26" t="inlineStr">
         <is>
           <t>Ben Van Don, P. Vinh Hoi, Q.4</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="20" t="inlineStr">
+      <c r="A44" s="26" t="inlineStr">
         <is>
           <t>River Gate</t>
         </is>
       </c>
-      <c r="B44" s="20" t="inlineStr">
+      <c r="B44" s="26" t="inlineStr">
         <is>
           <t>Q.4</t>
         </is>
       </c>
-      <c r="C44" s="20" t="n">
+      <c r="C44" s="26" t="n">
         <v>10.7626586</v>
       </c>
-      <c r="D44" s="20" t="n">
+      <c r="D44" s="26" t="n">
         <v>106.6991882</v>
       </c>
-      <c r="E44" s="20" t="inlineStr">
+      <c r="E44" s="26" t="inlineStr">
         <is>
           <t>3-4 ty</t>
         </is>
       </c>
-      <c r="F44" s="20" t="inlineStr">
+      <c r="F44" s="26" t="inlineStr">
         <is>
           <t>Ben Van Don, P. Khanh Hoi, Q.4</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="20" t="inlineStr">
+      <c r="A45" s="26" t="inlineStr">
         <is>
           <t>The Tresor</t>
         </is>
       </c>
-      <c r="B45" s="20" t="inlineStr">
+      <c r="B45" s="26" t="inlineStr">
         <is>
           <t>Q.4</t>
         </is>
       </c>
-      <c r="C45" s="20" t="n">
+      <c r="C45" s="26" t="n">
         <v>10.766733</v>
       </c>
-      <c r="D45" s="20" t="n">
+      <c r="D45" s="26" t="n">
         <v>106.7032221</v>
       </c>
-      <c r="E45" s="20" t="inlineStr">
+      <c r="E45" s="26" t="inlineStr">
         <is>
           <t>3.4 ty</t>
         </is>
       </c>
-      <c r="F45" s="20" t="inlineStr">
+      <c r="F45" s="26" t="inlineStr">
         <is>
           <t>Ben Van Don, P. Xom Chieu, Q.4</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="20" t="inlineStr">
+      <c r="A46" s="26" t="inlineStr">
         <is>
           <t>Q7 Saigon Riverside</t>
         </is>
       </c>
-      <c r="B46" s="20" t="inlineStr">
+      <c r="B46" s="26" t="inlineStr">
         <is>
           <t>Q.7</t>
         </is>
       </c>
-      <c r="C46" s="20" t="n">
+      <c r="C46" s="26" t="n">
         <v>10.7229238</v>
       </c>
-      <c r="D46" s="20" t="n">
+      <c r="D46" s="26" t="n">
         <v>106.7415437</v>
       </c>
-      <c r="E46" s="20" t="inlineStr">
+      <c r="E46" s="26" t="inlineStr">
         <is>
           <t>3.1-3.6 ty</t>
         </is>
       </c>
-      <c r="F46" s="20" t="inlineStr">
+      <c r="F46" s="26" t="inlineStr">
         <is>
           <t>Dao Tri, P. Phu Thuan, Q.7</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="20" t="inlineStr">
+      <c r="A47" s="26" t="inlineStr">
         <is>
           <t>Luxcity</t>
         </is>
       </c>
-      <c r="B47" s="20" t="inlineStr">
+      <c r="B47" s="26" t="inlineStr">
         <is>
           <t>Q.7</t>
         </is>
       </c>
-      <c r="C47" s="20" t="n">
+      <c r="C47" s="26" t="n">
         <v>10.7387122</v>
       </c>
-      <c r="D47" s="20" t="n">
+      <c r="D47" s="26" t="n">
         <v>106.7299709</v>
       </c>
-      <c r="E47" s="20" t="inlineStr">
+      <c r="E47" s="26" t="inlineStr">
         <is>
           <t>4.3-5 ty</t>
         </is>
       </c>
-      <c r="F47" s="20" t="inlineStr">
+      <c r="F47" s="26" t="inlineStr">
         <is>
           <t>Huynh Tan Phat, P. Binh Thuan, Q.7</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="20" t="inlineStr">
+      <c r="A48" s="26" t="inlineStr">
         <is>
           <t>River Panorama</t>
         </is>
       </c>
-      <c r="B48" s="20" t="inlineStr">
+      <c r="B48" s="26" t="inlineStr">
         <is>
           <t>Q.7</t>
         </is>
       </c>
-      <c r="C48" s="20" t="n">
+      <c r="C48" s="26" t="n">
         <v>10.7145604</v>
       </c>
-      <c r="D48" s="20" t="n">
+      <c r="D48" s="26" t="n">
         <v>106.7415783</v>
       </c>
-      <c r="E48" s="20" t="inlineStr">
+      <c r="E48" s="26" t="inlineStr">
         <is>
           <t>3.9-4.7 ty</t>
         </is>
       </c>
-      <c r="F48" s="20" t="inlineStr">
+      <c r="F48" s="26" t="inlineStr">
         <is>
           <t>Hoang Quoc Viet, P. Phu Thuan, Q.7</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="20" t="inlineStr">
+      <c r="A49" s="26" t="inlineStr">
         <is>
           <t>Q7 Boulevard</t>
         </is>
       </c>
-      <c r="B49" s="20" t="inlineStr">
+      <c r="B49" s="26" t="inlineStr">
         <is>
           <t>Q.7</t>
         </is>
       </c>
-      <c r="C49" s="20" t="n">
+      <c r="C49" s="26" t="n">
         <v>10.7078219</v>
       </c>
-      <c r="D49" s="20" t="n">
+      <c r="D49" s="26" t="n">
         <v>106.7329454</v>
       </c>
-      <c r="E49" s="20" t="inlineStr">
+      <c r="E49" s="26" t="inlineStr">
         <is>
           <t>3.3-3.9 ty</t>
         </is>
       </c>
-      <c r="F49" s="20" t="inlineStr">
+      <c r="F49" s="26" t="inlineStr">
         <is>
           <t>Nguyen Luong Bang, P. Phu My, Q.7</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="20" t="inlineStr">
+      <c r="A50" s="26" t="inlineStr">
         <is>
           <t>Sunshine Sky City</t>
         </is>
       </c>
-      <c r="B50" s="20" t="inlineStr">
+      <c r="B50" s="26" t="inlineStr">
         <is>
           <t>Q.7</t>
         </is>
       </c>
-      <c r="C50" s="20" t="n">
+      <c r="C50" s="26" t="n">
         <v>10.7295023</v>
       </c>
-      <c r="D50" s="20" t="n">
+      <c r="D50" s="26" t="n">
         <v>106.7304584</v>
       </c>
-      <c r="E50" s="20" t="inlineStr">
+      <c r="E50" s="26" t="inlineStr">
         <is>
           <t>4.2 ty</t>
         </is>
       </c>
-      <c r="F50" s="20" t="inlineStr">
+      <c r="F50" s="26" t="inlineStr">
         <is>
           <t>Phu Thuan, P. Tan Phu, Q.7</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="20" t="inlineStr">
+      <c r="A51" s="26" t="inlineStr">
         <is>
           <t>Eco Green Sai Gon</t>
         </is>
       </c>
-      <c r="B51" s="20" t="inlineStr">
+      <c r="B51" s="26" t="inlineStr">
         <is>
           <t>Q.7</t>
         </is>
       </c>
-      <c r="C51" s="20" t="n">
+      <c r="C51" s="26" t="n">
         <v>10.7487183</v>
       </c>
-      <c r="D51" s="20" t="n">
+      <c r="D51" s="26" t="n">
         <v>106.723741</v>
       </c>
-      <c r="E51" s="20" t="inlineStr">
+      <c r="E51" s="26" t="inlineStr">
         <is>
           <t>4.8-5 ty</t>
         </is>
       </c>
-      <c r="F51" s="20" t="inlineStr">
+      <c r="F51" s="26" t="inlineStr">
         <is>
           <t>Nguyen Van Linh, P. Tan Thuan Tay, Q.7</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="20" t="inlineStr">
+      <c r="A52" s="26" t="inlineStr">
         <is>
           <t>Jamona City</t>
         </is>
       </c>
-      <c r="B52" s="20" t="inlineStr">
+      <c r="B52" s="26" t="inlineStr">
         <is>
           <t>Q.7</t>
         </is>
       </c>
-      <c r="C52" s="20" t="n">
+      <c r="C52" s="26" t="n">
         <v>10.737552</v>
       </c>
-      <c r="D52" s="20" t="n">
+      <c r="D52" s="26" t="n">
         <v>106.7374244</v>
       </c>
-      <c r="E52" s="20" t="inlineStr">
+      <c r="E52" s="26" t="inlineStr">
         <is>
           <t>3-3.4 ty</t>
         </is>
       </c>
-      <c r="F52" s="20" t="inlineStr">
+      <c r="F52" s="26" t="inlineStr">
         <is>
           <t>Dao Tri, P. Phu Thuan, Q.7</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="20" t="inlineStr">
+      <c r="A53" s="26" t="inlineStr">
         <is>
           <t>Sunrise City</t>
         </is>
       </c>
-      <c r="B53" s="20" t="inlineStr">
+      <c r="B53" s="26" t="inlineStr">
         <is>
           <t>Q.7</t>
         </is>
       </c>
-      <c r="C53" s="20" t="n">
+      <c r="C53" s="26" t="n">
         <v>10.7437289</v>
       </c>
-      <c r="D53" s="20" t="n">
+      <c r="D53" s="26" t="n">
         <v>106.7011024</v>
       </c>
-      <c r="E53" s="20" t="inlineStr">
+      <c r="E53" s="26" t="inlineStr">
         <is>
           <t>3.3 ty</t>
         </is>
       </c>
-      <c r="F53" s="20" t="inlineStr">
+      <c r="F53" s="26" t="inlineStr">
         <is>
           <t>Nguyen Huu Tho, P. Tan Hung, Q.7</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="20" t="inlineStr">
+      <c r="A54" s="26" t="inlineStr">
         <is>
           <t>The Era Town</t>
         </is>
       </c>
-      <c r="B54" s="20" t="inlineStr">
+      <c r="B54" s="26" t="inlineStr">
         <is>
           <t>Q.7</t>
         </is>
       </c>
-      <c r="C54" s="20" t="n">
+      <c r="C54" s="26" t="n">
         <v>10.7000497</v>
       </c>
-      <c r="D54" s="20" t="n">
+      <c r="D54" s="26" t="n">
         <v>106.7330581</v>
       </c>
-      <c r="E54" s="20" t="inlineStr">
+      <c r="E54" s="26" t="inlineStr">
         <is>
           <t>3.3 ty</t>
         </is>
       </c>
-      <c r="F54" s="20" t="inlineStr">
+      <c r="F54" s="26" t="inlineStr">
         <is>
           <t>P. Phu My, Q.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="26" t="inlineStr">
+        <is>
+          <t>The Origami (Vinhomes Grand Park)</t>
+        </is>
+      </c>
+      <c r="B55" s="26" t="inlineStr">
+        <is>
+          <t>Q.9</t>
+        </is>
+      </c>
+      <c r="C55" s="26" t="n">
+        <v>10.8452092</v>
+      </c>
+      <c r="D55" s="26" t="n">
+        <v>106.8378812</v>
+      </c>
+      <c r="E55" s="26" t="inlineStr">
+        <is>
+          <t>3.3-4.9 ty</t>
+        </is>
+      </c>
+      <c r="F55" s="26" t="inlineStr">
+        <is>
+          <t>Long Binh, TP.Thu Duc (Q.9 cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="26" t="inlineStr">
+        <is>
+          <t>Lumiere Boulevard</t>
+        </is>
+      </c>
+      <c r="B56" s="26" t="inlineStr">
+        <is>
+          <t>Q.9</t>
+        </is>
+      </c>
+      <c r="C56" s="26" t="n">
+        <v>10.8394996</v>
+      </c>
+      <c r="D56" s="26" t="n">
+        <v>106.8392649</v>
+      </c>
+      <c r="E56" s="26" t="inlineStr">
+        <is>
+          <t>4.6-4.7 ty</t>
+        </is>
+      </c>
+      <c r="F56" s="26" t="inlineStr">
+        <is>
+          <t>Long Binh, TP.Thu Duc (Q.9 cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="26" t="inlineStr">
+        <is>
+          <t>Mizuki Park</t>
+        </is>
+      </c>
+      <c r="B57" s="26" t="inlineStr">
+        <is>
+          <t>Binh Chanh</t>
+        </is>
+      </c>
+      <c r="C57" s="26" t="n">
+        <v>10.7152713</v>
+      </c>
+      <c r="D57" s="26" t="n">
+        <v>106.6634002</v>
+      </c>
+      <c r="E57" s="26" t="inlineStr">
+        <is>
+          <t>3.6-4.2 ty</t>
+        </is>
+      </c>
+      <c r="F57" s="26" t="inlineStr">
+        <is>
+          <t>Nguyen Van Linh, X.Binh Hung, Binh Chanh</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="26" t="inlineStr">
+        <is>
+          <t>Trellia Cove (Mizuki Park)</t>
+        </is>
+      </c>
+      <c r="B58" s="26" t="inlineStr">
+        <is>
+          <t>Binh Chanh</t>
+        </is>
+      </c>
+      <c r="C58" s="26" t="n">
+        <v>10.7128997</v>
+      </c>
+      <c r="D58" s="26" t="n">
+        <v>106.6607158</v>
+      </c>
+      <c r="E58" s="26" t="inlineStr">
+        <is>
+          <t>3.9-5 ty</t>
+        </is>
+      </c>
+      <c r="F58" s="26" t="inlineStr">
+        <is>
+          <t>Nguyen Van Linh, X.Binh Hung, Binh Chanh</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="26" t="inlineStr">
+        <is>
+          <t>Westgate An Gia</t>
+        </is>
+      </c>
+      <c r="B59" s="26" t="inlineStr">
+        <is>
+          <t>Binh Chanh</t>
+        </is>
+      </c>
+      <c r="C59" s="26" t="n">
+        <v>10.6892919</v>
+      </c>
+      <c r="D59" s="26" t="n">
+        <v>106.5857392</v>
+      </c>
+      <c r="E59" s="26" t="inlineStr">
+        <is>
+          <t>3.2-4.5 ty</t>
+        </is>
+      </c>
+      <c r="F59" s="26" t="inlineStr">
+        <is>
+          <t>Nguyen Van Linh, TT.Tan Tuc, Binh Chanh</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="26" t="inlineStr">
+        <is>
+          <t>Sai Gon Mia</t>
+        </is>
+      </c>
+      <c r="B60" s="26" t="inlineStr">
+        <is>
+          <t>Binh Chanh</t>
+        </is>
+      </c>
+      <c r="C60" s="26" t="n">
+        <v>10.7326451</v>
+      </c>
+      <c r="D60" s="26" t="n">
+        <v>106.688988</v>
+      </c>
+      <c r="E60" s="26" t="inlineStr">
+        <is>
+          <t>3.4-5 ty</t>
+        </is>
+      </c>
+      <c r="F60" s="26" t="inlineStr">
+        <is>
+          <t>Trung Son, X.Binh Hung, Binh Chanh</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: lookup real coords via Nominatim for Tan Phu/Binh/Binh Chanh projects
- Cleaned 14 project names (Hung 1/Phu 4/Ky/Thanh URL-slug prefixes -> bare project names)
- OSM Nominatim API lookup for 39 candidate projects (within target districts, clean names)
- 26 hits via name+district queries
- Validated against district polygons; restored 6 false matches (Phuc Yen, Carillon 7, An Gia Garden, etc. that Nominatim sent to wrong district)
- Reparented 8 sub-projects (Diamond Centery/Emerald/Ruby/Alnata Plus/Brilliant/The Glen -> Celadon City; Trellia Cove -> Mizuki Park) with small jitter

Major real coords now: Mizuki Park, Celadon City complex, Botanica Premier, Sky Center, Park Legend, Sai Gon Airport Plaza, RichStar, Lotus Garden, HQC Plaza, Lovera Vista, etc.
</commit_message>
<xml_diff>
--- a/chung_cu_data.xlsx
+++ b/chung_cu_data.xlsx
@@ -796,7 +796,7 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Phu 4 Sai Gon Intela</t>
+          <t>Sai Gon Intela</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Phu 4 Lovera Vista</t>
+          <t>Lovera Vista</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Thanh Investco Babylon</t>
+          <t>Investco Babylon</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Phu 4 Terra Luxury</t>
+          <t>Terra Luxury</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -2943,7 +2943,7 @@
       </c>
       <c r="B35" s="17" t="inlineStr">
         <is>
-          <t>Res 11</t>
+          <t>RES 11</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Thanh 70</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Ky Diamond Alnata</t>
+          <t>Diamond Alnata</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Ky Tanibuilding Son Ky 2</t>
+          <t>Tanibuilding Son Ky 2</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -4385,7 +4385,7 @@
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Hung 1 Mizuki Park</t>
+          <t>Mizuki Park</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -4450,7 +4450,7 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Hung 1 Trellia Cove</t>
+          <t>Trellia Cove</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -4803,7 +4803,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Ky 70</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Hung 1 Sai Gon Mia</t>
+          <t>Sai Gon Mia</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Tho Hoa Fortuna Vuon Lai</t>
+          <t>Fortuna Vuon Lai</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -5997,7 +5997,7 @@
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Phu Tay Hqc Plaza</t>
+          <t>HQC Plaza</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -6255,10 +6255,10 @@
         </is>
       </c>
       <c r="C2" s="20" t="n">
-        <v>10.7729244</v>
+        <v>10.7727625</v>
       </c>
       <c r="D2" s="20" t="n">
-        <v>106.6257607</v>
+        <v>106.6267493</v>
       </c>
       <c r="E2" s="20" t="inlineStr">
         <is>
@@ -6283,10 +6283,10 @@
         </is>
       </c>
       <c r="C3" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.813</v>
       </c>
       <c r="D3" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.65884</v>
       </c>
       <c r="E3" s="20" t="inlineStr">
         <is>
@@ -6302,7 +6302,7 @@
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t>Phu 4 Sai Gon Intela</t>
+          <t>Sai Gon Intela</t>
         </is>
       </c>
       <c r="B4" s="20" t="inlineStr">
@@ -6311,10 +6311,10 @@
         </is>
       </c>
       <c r="C4" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.7243911</v>
       </c>
       <c r="D4" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.5986942</v>
       </c>
       <c r="E4" s="20" t="inlineStr">
         <is>
@@ -6330,7 +6330,7 @@
     <row r="5">
       <c r="A5" s="20" t="inlineStr">
         <is>
-          <t>Phu 4 Lovera Vista</t>
+          <t>Lovera Vista</t>
         </is>
       </c>
       <c r="B5" s="20" t="inlineStr">
@@ -6339,10 +6339,10 @@
         </is>
       </c>
       <c r="C5" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.6919182</v>
       </c>
       <c r="D5" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.6422011</v>
       </c>
       <c r="E5" s="20" t="inlineStr">
         <is>
@@ -6367,10 +6367,10 @@
         </is>
       </c>
       <c r="C6" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.7210978</v>
       </c>
       <c r="D6" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.5926648</v>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
@@ -6498,7 +6498,7 @@
     <row r="11">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>Thanh Investco Babylon</t>
+          <t>Investco Babylon</t>
         </is>
       </c>
       <c r="B11" s="20" t="inlineStr">
@@ -6507,10 +6507,10 @@
         </is>
       </c>
       <c r="C11" s="20" t="n">
-        <v>10.78728571428571</v>
+        <v>10.7889462</v>
       </c>
       <c r="D11" s="20" t="n">
-        <v>106.6278904761905</v>
+        <v>106.6398628</v>
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
@@ -6535,10 +6535,10 @@
         </is>
       </c>
       <c r="C12" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.8109666</v>
       </c>
       <c r="D12" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6599382</v>
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
@@ -6563,10 +6563,10 @@
         </is>
       </c>
       <c r="C13" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.805859</v>
       </c>
       <c r="D13" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6594014</v>
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
@@ -6582,7 +6582,7 @@
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>Phu 4 Terra Luxury</t>
+          <t>Terra Luxury</t>
         </is>
       </c>
       <c r="B14" s="20" t="inlineStr">
@@ -6591,10 +6591,10 @@
         </is>
       </c>
       <c r="C14" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.7222143</v>
       </c>
       <c r="D14" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.5979179</v>
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
@@ -6619,10 +6619,10 @@
         </is>
       </c>
       <c r="C15" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.7209096</v>
       </c>
       <c r="D15" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.5998253</v>
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         </is>
       </c>
       <c r="C16" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.7227706</v>
       </c>
       <c r="D16" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.5910702</v>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
@@ -6731,10 +6731,10 @@
         </is>
       </c>
       <c r="C19" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.8149357</v>
       </c>
       <c r="D19" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6662829</v>
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
@@ -6759,10 +6759,10 @@
         </is>
       </c>
       <c r="C20" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.8080296</v>
       </c>
       <c r="D20" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6633153</v>
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
@@ -6787,10 +6787,10 @@
         </is>
       </c>
       <c r="C21" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.8040983</v>
       </c>
       <c r="D21" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6579044</v>
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
@@ -6815,10 +6815,10 @@
         </is>
       </c>
       <c r="C22" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.8082178</v>
       </c>
       <c r="D22" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6561548</v>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
@@ -6843,10 +6843,10 @@
         </is>
       </c>
       <c r="C23" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.7965292</v>
       </c>
       <c r="D23" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6416853</v>
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
@@ -7170,7 +7170,7 @@
     <row r="35">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>Res 11</t>
+          <t>RES 11</t>
         </is>
       </c>
       <c r="B35" s="20" t="inlineStr">
@@ -7347,10 +7347,10 @@
         </is>
       </c>
       <c r="C41" s="20" t="n">
-        <v>10.8009934</v>
+        <v>10.8025753</v>
       </c>
       <c r="D41" s="20" t="n">
-        <v>106.6129628</v>
+        <v>106.6147837</v>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
@@ -7375,10 +7375,10 @@
         </is>
       </c>
       <c r="C42" s="20" t="n">
-        <v>10.7961217</v>
+        <v>10.7963806</v>
       </c>
       <c r="D42" s="20" t="n">
-        <v>106.6366525</v>
+        <v>106.6370621</v>
       </c>
       <c r="E42" s="20" t="inlineStr">
         <is>
@@ -7403,10 +7403,10 @@
         </is>
       </c>
       <c r="C43" s="20" t="n">
-        <v>10.7742711</v>
+        <v>10.7736303</v>
       </c>
       <c r="D43" s="20" t="n">
-        <v>106.6357158</v>
+        <v>106.6356264</v>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
@@ -7431,10 +7431,10 @@
         </is>
       </c>
       <c r="C44" s="20" t="n">
-        <v>10.7776469</v>
+        <v>10.7776072</v>
       </c>
       <c r="D44" s="20" t="n">
-        <v>106.6369297</v>
+        <v>106.63697</v>
       </c>
       <c r="E44" s="20" t="inlineStr">
         <is>
@@ -7478,7 +7478,7 @@
     <row r="46">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>Thanh 70</t>
+          <t>70</t>
         </is>
       </c>
       <c r="B46" s="20" t="inlineStr">
@@ -7487,10 +7487,10 @@
         </is>
       </c>
       <c r="C46" s="20" t="n">
-        <v>10.78728571428571</v>
+        <v>10.7838094</v>
       </c>
       <c r="D46" s="20" t="n">
-        <v>106.6278904761905</v>
+        <v>106.6369877</v>
       </c>
       <c r="E46" s="20" t="inlineStr">
         <is>
@@ -7506,7 +7506,7 @@
     <row r="47">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>Ky Diamond Alnata</t>
+          <t>Diamond Alnata</t>
         </is>
       </c>
       <c r="B47" s="20" t="inlineStr">
@@ -7515,10 +7515,10 @@
         </is>
       </c>
       <c r="C47" s="20" t="n">
-        <v>10.78728571428571</v>
+        <v>10.8028969</v>
       </c>
       <c r="D47" s="20" t="n">
-        <v>106.6278904761905</v>
+        <v>106.6155408</v>
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
@@ -7534,7 +7534,7 @@
     <row r="48">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>Ky Tanibuilding Son Ky 2</t>
+          <t>Tanibuilding Son Ky 2</t>
         </is>
       </c>
       <c r="B48" s="20" t="inlineStr">
@@ -7543,10 +7543,10 @@
         </is>
       </c>
       <c r="C48" s="20" t="n">
-        <v>10.78728571428571</v>
+        <v>10.7832356</v>
       </c>
       <c r="D48" s="20" t="n">
-        <v>106.6278904761905</v>
+        <v>106.6259375</v>
       </c>
       <c r="E48" s="20" t="inlineStr">
         <is>
@@ -7571,10 +7571,10 @@
         </is>
       </c>
       <c r="C49" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.80625</v>
       </c>
       <c r="D49" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6549429</v>
       </c>
       <c r="E49" s="20" t="inlineStr">
         <is>
@@ -7599,10 +7599,10 @@
         </is>
       </c>
       <c r="C50" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.8053756</v>
       </c>
       <c r="D50" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6469127</v>
       </c>
       <c r="E50" s="20" t="inlineStr">
         <is>
@@ -7627,10 +7627,10 @@
         </is>
       </c>
       <c r="C51" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.72003</v>
       </c>
       <c r="D51" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.5976883</v>
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
@@ -7655,10 +7655,10 @@
         </is>
       </c>
       <c r="C52" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.7177394</v>
       </c>
       <c r="D52" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.597995</v>
       </c>
       <c r="E52" s="20" t="inlineStr">
         <is>
@@ -7683,10 +7683,10 @@
         </is>
       </c>
       <c r="C53" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.718739</v>
       </c>
       <c r="D53" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.5959114</v>
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
@@ -7711,10 +7711,10 @@
         </is>
       </c>
       <c r="C54" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.7191957</v>
       </c>
       <c r="D54" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.593763</v>
       </c>
       <c r="E54" s="20" t="inlineStr">
         <is>
@@ -7786,7 +7786,7 @@
     <row r="57">
       <c r="A57" s="20" t="inlineStr">
         <is>
-          <t>Hung 1 Mizuki Park</t>
+          <t>Mizuki Park</t>
         </is>
       </c>
       <c r="B57" s="20" t="inlineStr">
@@ -7795,10 +7795,10 @@
         </is>
       </c>
       <c r="C57" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.7143025</v>
       </c>
       <c r="D57" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.6624699</v>
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
@@ -7814,7 +7814,7 @@
     <row r="58">
       <c r="A58" s="20" t="inlineStr">
         <is>
-          <t>Hung 1 Trellia Cove</t>
+          <t>Trellia Cove</t>
         </is>
       </c>
       <c r="B58" s="20" t="inlineStr">
@@ -7823,10 +7823,10 @@
         </is>
       </c>
       <c r="C58" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.7139913</v>
       </c>
       <c r="D58" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.6623822</v>
       </c>
       <c r="E58" s="20" t="inlineStr">
         <is>
@@ -7851,10 +7851,10 @@
         </is>
       </c>
       <c r="C59" s="20" t="n">
-        <v>10.8022839</v>
+        <v>10.8021735</v>
       </c>
       <c r="D59" s="20" t="n">
-        <v>106.6158704</v>
+        <v>106.615341</v>
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
@@ -7879,10 +7879,10 @@
         </is>
       </c>
       <c r="C60" s="20" t="n">
-        <v>10.8053889</v>
+        <v>10.8019565</v>
       </c>
       <c r="D60" s="20" t="n">
-        <v>106.6148485</v>
+        <v>106.6146748</v>
       </c>
       <c r="E60" s="20" t="inlineStr">
         <is>
@@ -7907,10 +7907,10 @@
         </is>
       </c>
       <c r="C61" s="20" t="n">
-        <v>10.8028716</v>
+        <v>10.8026957</v>
       </c>
       <c r="D61" s="20" t="n">
-        <v>106.615476</v>
+        <v>106.6147149</v>
       </c>
       <c r="E61" s="20" t="inlineStr">
         <is>
@@ -7935,10 +7935,10 @@
         </is>
       </c>
       <c r="C62" s="20" t="n">
-        <v>10.7896245</v>
+        <v>10.7895653</v>
       </c>
       <c r="D62" s="20" t="n">
-        <v>106.6394598</v>
+        <v>106.6393649</v>
       </c>
       <c r="E62" s="20" t="inlineStr">
         <is>
@@ -7954,7 +7954,7 @@
     <row r="63">
       <c r="A63" s="20" t="inlineStr">
         <is>
-          <t>Ky 70</t>
+          <t>70</t>
         </is>
       </c>
       <c r="B63" s="20" t="inlineStr">
@@ -7963,10 +7963,10 @@
         </is>
       </c>
       <c r="C63" s="20" t="n">
-        <v>10.78728571428571</v>
+        <v>10.7838094</v>
       </c>
       <c r="D63" s="20" t="n">
-        <v>106.6278904761905</v>
+        <v>106.6369877</v>
       </c>
       <c r="E63" s="20" t="inlineStr">
         <is>
@@ -7991,10 +7991,10 @@
         </is>
       </c>
       <c r="C64" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.8062382</v>
       </c>
       <c r="D64" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6662711</v>
       </c>
       <c r="E64" s="20" t="inlineStr">
         <is>
@@ -8019,10 +8019,10 @@
         </is>
       </c>
       <c r="C65" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.8000536</v>
       </c>
       <c r="D65" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6651001</v>
       </c>
       <c r="E65" s="20" t="inlineStr">
         <is>
@@ -8038,7 +8038,7 @@
     <row r="66">
       <c r="A66" s="20" t="inlineStr">
         <is>
-          <t>Hung 1 Sai Gon Mia</t>
+          <t>Sai Gon Mia</t>
         </is>
       </c>
       <c r="B66" s="20" t="inlineStr">
@@ -8047,10 +8047,10 @@
         </is>
       </c>
       <c r="C66" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.7231867</v>
       </c>
       <c r="D66" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.5933435</v>
       </c>
       <c r="E66" s="20" t="inlineStr">
         <is>
@@ -8243,10 +8243,10 @@
         </is>
       </c>
       <c r="C73" s="20" t="n">
-        <v>10.803599</v>
+        <v>10.8025777</v>
       </c>
       <c r="D73" s="20" t="n">
-        <v>106.6188954</v>
+        <v>106.614893</v>
       </c>
       <c r="E73" s="20" t="inlineStr">
         <is>
@@ -8271,10 +8271,10 @@
         </is>
       </c>
       <c r="C74" s="20" t="n">
-        <v>10.803923</v>
+        <v>10.8020962</v>
       </c>
       <c r="D74" s="20" t="n">
-        <v>106.6152349</v>
+        <v>106.614808</v>
       </c>
       <c r="E74" s="20" t="inlineStr">
         <is>
@@ -8299,10 +8299,10 @@
         </is>
       </c>
       <c r="C75" s="20" t="n">
-        <v>10.8020447</v>
+        <v>10.8023127</v>
       </c>
       <c r="D75" s="20" t="n">
-        <v>106.6145601</v>
+        <v>106.6142934</v>
       </c>
       <c r="E75" s="20" t="inlineStr">
         <is>
@@ -8318,7 +8318,7 @@
     <row r="76">
       <c r="A76" s="20" t="inlineStr">
         <is>
-          <t>Tho Hoa Fortuna Vuon Lai</t>
+          <t>Fortuna Vuon Lai</t>
         </is>
       </c>
       <c r="B76" s="20" t="inlineStr">
@@ -8327,10 +8327,10 @@
         </is>
       </c>
       <c r="C76" s="20" t="n">
-        <v>10.78728571428571</v>
+        <v>10.7883906</v>
       </c>
       <c r="D76" s="20" t="n">
-        <v>106.6278904761905</v>
+        <v>106.6244178</v>
       </c>
       <c r="E76" s="20" t="inlineStr">
         <is>
@@ -8355,10 +8355,10 @@
         </is>
       </c>
       <c r="C77" s="20" t="n">
-        <v>10.78728571428571</v>
+        <v>10.7900957</v>
       </c>
       <c r="D77" s="20" t="n">
-        <v>106.6278904761905</v>
+        <v>106.6243718</v>
       </c>
       <c r="E77" s="20" t="inlineStr">
         <is>
@@ -8383,10 +8383,10 @@
         </is>
       </c>
       <c r="C78" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.8115758</v>
       </c>
       <c r="D78" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.669586</v>
       </c>
       <c r="E78" s="20" t="inlineStr">
         <is>
@@ -8411,10 +8411,10 @@
         </is>
       </c>
       <c r="C79" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.7909</v>
       </c>
       <c r="D79" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6457395</v>
       </c>
       <c r="E79" s="20" t="inlineStr">
         <is>
@@ -8439,10 +8439,10 @@
         </is>
       </c>
       <c r="C80" s="20" t="n">
-        <v>10.8085</v>
+        <v>10.812611</v>
       </c>
       <c r="D80" s="20" t="n">
-        <v>106.6588411764706</v>
+        <v>106.6570097</v>
       </c>
       <c r="E80" s="20" t="inlineStr">
         <is>
@@ -8458,7 +8458,7 @@
     <row r="81">
       <c r="A81" s="20" t="inlineStr">
         <is>
-          <t>Phu Tay Hqc Plaza</t>
+          <t>HQC Plaza</t>
         </is>
       </c>
       <c r="B81" s="20" t="inlineStr">
@@ -8467,10 +8467,10 @@
         </is>
       </c>
       <c r="C81" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.6945666</v>
       </c>
       <c r="D81" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.6063942</v>
       </c>
       <c r="E81" s="20" t="inlineStr">
         <is>
@@ -8495,10 +8495,10 @@
         </is>
       </c>
       <c r="C82" s="20" t="n">
-        <v>10.72137647058823</v>
+        <v>10.725491</v>
       </c>
       <c r="D82" s="20" t="n">
-        <v>106.5953529411765</v>
+        <v>106.5935197</v>
       </c>
       <c r="E82" s="20" t="inlineStr">
         <is>

</xml_diff>